<commit_message>
extract excel sheet data test
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a60af247b9013c15/codes_od/new_search_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:1_{0F46C67D-B5ED-4D4B-8A9D-78C816927189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13C3FB03-CEAF-4D7B-8531-183CD9916FA0}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="13_ncr:1_{0F46C67D-B5ED-4D4B-8A9D-78C816927189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D6EB423-1BAE-4E9D-B1CC-48447933CBA6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="タイトル行ありSh(3)" sheetId="3" r:id="rId1"/>
-    <sheet name="品名１列Sh(4)" sheetId="4" r:id="rId2"/>
+    <sheet name="タイトル行ありSh(4)" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="26">
   <si>
     <t>備考</t>
     <rPh sb="0" eb="2">
@@ -61,13 +61,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>P・G名</t>
-    <rPh sb="3" eb="4">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>数量</t>
     <rPh sb="0" eb="2">
       <t>スウリョウ</t>
@@ -137,14 +130,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>ｓｓ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ｇｇｇ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>さあｓ</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -156,31 +141,30 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>うぇああうぇｒ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ｆｓｄｆｄｓ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ｊｊｊ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ｄｌｌｌｌ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>れてｒ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>５５えｒｔれ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ｄｄｓｆｔ</t>
+    <t>PG名</t>
+    <rPh sb="2" eb="3">
+      <t>メイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>２列目１</t>
+    <rPh sb="1" eb="2">
+      <t>レツ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>メ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>２列目２</t>
+    <rPh sb="1" eb="2">
+      <t>レツ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>メ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -265,19 +249,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -295,6 +282,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -564,19 +555,29 @@
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="9.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="A1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
@@ -585,15 +586,15 @@
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="4"/>
+      <c r="C3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="6"/>
       <c r="E3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>0</v>
@@ -605,11 +606,11 @@
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F4" s="1">
         <v>1</v>
@@ -628,10 +629,10 @@
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>3</v>
@@ -642,10 +643,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -662,11 +663,11 @@
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
@@ -679,17 +680,17 @@
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" s="1">
         <v>5</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -699,10 +700,10 @@
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -714,16 +715,16 @@
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F10" s="1">
         <v>3</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -732,19 +733,19 @@
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="C3:D3"/>
-    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -752,7 +753,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC4DCD5-F5D9-434B-9150-22CA2C460DB7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74AF9B51-FD32-4D25-94B3-81B9E59CB18B}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
@@ -761,14 +762,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
+      <c r="A1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
@@ -777,14 +786,14 @@
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
+      <c r="C3" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>0</v>
@@ -796,10 +805,10 @@
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
@@ -814,13 +823,13 @@
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>3</v>
@@ -831,10 +840,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1">
@@ -850,10 +859,10 @@
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E7" s="1">
         <v>0</v>
@@ -866,16 +875,16 @@
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" s="1">
         <v>5</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -883,11 +892,9 @@
         <v>6</v>
       </c>
       <c r="B9" s="1"/>
-      <c r="C9" s="1" t="s">
-        <v>31</v>
-      </c>
+      <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -897,17 +904,15 @@
         <v>7</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="C10" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="C10" s="1"/>
       <c r="D10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" s="1">
         <v>3</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -916,10 +921,10 @@
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>

</xml_diff>